<commit_message>
updated music control to not necessary
</commit_message>
<xml_diff>
--- a/mcmods.xlsx
+++ b/mcmods.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Wichtig?</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>continuity</t>
+  </si>
+  <si>
+    <t>nicht mehr benötigt</t>
   </si>
 </sst>
 </file>
@@ -201,7 +204,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,6 +232,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor rgb="FFC55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor rgb="FF993300"/>
       </patternFill>
     </fill>
@@ -260,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -277,6 +292,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -628,6 +645,9 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
+      <c r="I7" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
@@ -836,7 +856,7 @@
       <c r="D24" s="7"/>
       <c r="E24" s="7"/>
       <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="G24" s="13"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>

</xml_diff>

<commit_message>
Updated to 26.2 only betterF3 missing
</commit_message>
<xml_diff>
--- a/mcmods.xlsx
+++ b/mcmods.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
   <si>
     <t>Wichtig?</t>
   </si>
@@ -146,9 +146,6 @@
     <t>immediatly fast</t>
   </si>
   <si>
-    <t>ferritcore</t>
-  </si>
-  <si>
     <t>shulkerbox tooltip</t>
   </si>
   <si>
@@ -162,13 +159,19 @@
   </si>
   <si>
     <t>*26.1.2</t>
+  </si>
+  <si>
+    <t>*26.2</t>
+  </si>
+  <si>
+    <t>ferritecore</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,8 +209,15 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -248,12 +258,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor rgb="FF993300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
-        <bgColor rgb="FF339966"/>
       </patternFill>
     </fill>
     <fill>
@@ -315,10 +319,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -580,16 +584,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:J67"/>
+  <dimension ref="A3:N67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
     <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" customWidth="1"/>
+    <col min="14" max="14" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -611,14 +616,17 @@
       <c r="G3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
@@ -630,12 +638,13 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
-      <c r="H4" s="14"/>
-      <c r="J4" s="7" t="s">
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="N4" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -648,11 +657,12 @@
       <c r="F5" s="7"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
-      <c r="J5" s="8" t="s">
+      <c r="I5" s="8"/>
+      <c r="N5" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6" t="s">
         <v>37</v>
@@ -663,11 +673,12 @@
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
-      <c r="J6" s="9" t="s">
+      <c r="I6" s="7"/>
+      <c r="N6" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="6" t="s">
         <v>13</v>
@@ -678,11 +689,12 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
-      <c r="J7" s="12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I7" s="7"/>
+      <c r="N7" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
@@ -695,8 +707,9 @@
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I8" s="7"/>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="6" t="s">
         <v>16</v>
@@ -707,8 +720,9 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
-    </row>
-    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I9" s="8"/>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
@@ -721,11 +735,12 @@
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -733,8 +748,9 @@
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I11" s="7"/>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>8</v>
       </c>
@@ -747,8 +763,9 @@
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I12" s="7"/>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="6" t="s">
         <v>38</v>
@@ -759,8 +776,9 @@
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I13" s="7"/>
+    </row>
+    <row r="14" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>8</v>
       </c>
@@ -773,8 +791,9 @@
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
@@ -787,13 +806,14 @@
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
-    </row>
-    <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
@@ -801,8 +821,9 @@
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I16" s="7"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>8</v>
       </c>
@@ -815,8 +836,9 @@
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I17" s="7"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>8</v>
       </c>
@@ -829,8 +851,9 @@
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="6" t="s">
         <v>22</v>
@@ -840,9 +863,10 @@
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>8</v>
       </c>
@@ -855,8 +879,9 @@
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>8</v>
       </c>
@@ -869,8 +894,9 @@
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>8</v>
       </c>
@@ -883,8 +909,9 @@
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="6" t="s">
         <v>26</v>
@@ -895,8 +922,9 @@
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I23" s="7"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="6" t="s">
         <v>27</v>
@@ -906,12 +934,13 @@
       <c r="E24" s="7"/>
       <c r="F24" s="8"/>
       <c r="G24" s="13"/>
-      <c r="H24" s="17"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
@@ -919,11 +948,12 @@
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I25" s="7"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
@@ -931,8 +961,9 @@
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I26" s="7"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>8</v>
       </c>
@@ -945,8 +976,9 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I27" s="7"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>8</v>
       </c>
@@ -959,8 +991,9 @@
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I28" s="7"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>8</v>
       </c>
@@ -973,8 +1006,9 @@
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I29" s="7"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="6" t="s">
         <v>31</v>
@@ -985,8 +1019,9 @@
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I30" s="7"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="6" t="s">
         <v>32</v>
@@ -997,8 +1032,9 @@
       <c r="F31" s="7"/>
       <c r="G31" s="11"/>
       <c r="H31" s="11"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I31" s="11"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>8</v>
       </c>
@@ -1011,8 +1047,9 @@
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I32" s="7"/>
+    </row>
+    <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>8</v>
       </c>
@@ -1025,8 +1062,9 @@
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I33" s="7"/>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>8</v>
       </c>
@@ -1039,8 +1077,9 @@
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I34" s="7"/>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>8</v>
       </c>
@@ -1053,6 +1092,7 @@
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C67">

</xml_diff>

<commit_message>
added mods for 26.3
</commit_message>
<xml_diff>
--- a/mcmods.xlsx
+++ b/mcmods.xlsx
@@ -744,7 +744,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="10"/>
+      <c r="J7" s="8"/>
       <c r="N7" s="13" t="s">
         <v>19</v>
       </c>
@@ -837,7 +837,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
-      <c r="J13" s="10"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">

</xml_diff>

<commit_message>
added MiniHUD and Malilib and updated to newest fabric api
</commit_message>
<xml_diff>
--- a/mcmods.xlsx
+++ b/mcmods.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="50">
   <si>
     <t xml:space="preserve">Wichtig?</t>
   </si>
@@ -122,6 +122,12 @@
   </si>
   <si>
     <t xml:space="preserve">lithium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malilib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minihud</t>
   </si>
   <si>
     <t xml:space="preserve">modmenu</t>
@@ -634,7 +640,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A3:N67"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.71"/>
@@ -993,7 +999,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
-      <c r="J23" s="15"/>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
@@ -1003,11 +1009,11 @@
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6"/>
@@ -1021,7 +1027,7 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
+      <c r="J25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6"/>
@@ -1031,11 +1037,11 @@
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
@@ -1106,7 +1112,7 @@
       </c>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
-      <c r="E31" s="16"/>
+      <c r="E31" s="8"/>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -1138,7 +1144,7 @@
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="E33" s="16"/>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
@@ -1176,6 +1182,32 @@
       <c r="H35" s="8"/>
       <c r="I35" s="8"/>
       <c r="J35" s="8"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="1" t="n">

</xml_diff>